<commit_message>
Update today's file: 26????????\26????????\????&?????\????.20260302.xlsx
</commit_message>
<xml_diff>
--- a/26年信息化项目资料/26年信息化项目资料/事项记录&风险记录表/事项梳理.20260302.xlsx
+++ b/26年信息化项目资料/26年信息化项目资料/事项记录&风险记录表/事项梳理.20260302.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="304">
   <si>
     <t>山东省创新发展研究院电话号码表</t>
   </si>
@@ -782,6 +782,9 @@
   </si>
   <si>
     <t>《关于山东省科技成果“以演代评”“以演促转”数字平台解决方案》</t>
+  </si>
+  <si>
+    <t>成浩，项目有后续情况后同步</t>
   </si>
   <si>
     <t>26年实施方案</t>
@@ -54672,7 +54675,9 @@
       <c r="D44" s="40"/>
       <c r="E44" s="40"/>
       <c r="F44" s="40"/>
-      <c r="G44" s="40"/>
+      <c r="G44" s="40" t="s">
+        <v>243</v>
+      </c>
       <c r="H44" s="40"/>
       <c r="I44" s="40"/>
       <c r="J44" s="40"/>
@@ -71065,28 +71070,28 @@
     </row>
     <row r="46" ht="21" spans="1:1024 1025:16384">
       <c r="A46" s="73" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B46" s="75"/>
     </row>
     <row r="47" spans="1:1024 1025:16384">
       <c r="B47" s="22" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="48" spans="1:1024 1025:16384">
       <c r="B48" s="22" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="B49" s="22" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="B50" s="22" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -71208,45 +71213,45 @@
   <sheetData>
     <row r="1" spans="1:24">
       <c r="A1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:24">
       <c r="B3" s="4"/>
       <c r="C3" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H3" s="10"/>
       <c r="I3" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:24">
       <c r="B4" s="7" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>138</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="7" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F4" s="10"/>
       <c r="G4" s="7" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H4" s="10"/>
       <c r="I4" s="7" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="T4" s="12"/>
       <c r="U4" s="12"/>
@@ -71265,7 +71270,7 @@
       <c r="G5" s="7"/>
       <c r="H5" s="10"/>
       <c r="I5" s="7" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="T5" s="12"/>
       <c r="U5" s="12"/>
@@ -71284,7 +71289,7 @@
       <c r="G6" s="7"/>
       <c r="H6" s="10"/>
       <c r="I6" s="7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="T6" s="12"/>
       <c r="U6" s="12"/>
@@ -71309,22 +71314,22 @@
     </row>
     <row r="8" spans="1:24">
       <c r="B8" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>155</v>
       </c>
       <c r="D8" s="10"/>
       <c r="E8" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F8" s="10"/>
       <c r="G8" s="7" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H8" s="10"/>
       <c r="I8" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="T8" s="12"/>
       <c r="U8" s="12"/>
@@ -71341,7 +71346,7 @@
       <c r="G9" s="7"/>
       <c r="H9" s="10"/>
       <c r="I9" s="7" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="T9" s="12"/>
       <c r="U9" s="12"/>
@@ -71358,7 +71363,7 @@
       <c r="G10" s="7"/>
       <c r="H10" s="10"/>
       <c r="I10" s="7" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="T10" s="12"/>
       <c r="U10" s="12"/>
@@ -71378,22 +71383,22 @@
     </row>
     <row r="12" s="4" customFormat="1" spans="1:24">
       <c r="B12" s="7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F12" s="10"/>
       <c r="G12" s="7" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H12" s="10"/>
       <c r="I12" s="7" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="T12" s="14"/>
       <c r="U12" s="14"/>
@@ -71409,15 +71414,15 @@
     </row>
     <row r="14" spans="1:24">
       <c r="B14" s="7" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D14" s="13"/>
       <c r="F14" s="15"/>
       <c r="G14" s="16" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H14" s="13"/>
     </row>
@@ -71425,7 +71430,7 @@
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="G15" s="7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -71462,7 +71467,7 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -71483,64 +71488,64 @@
         <v>125</v>
       </c>
       <c r="B2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" spans="1:14">
       <c r="B3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:14">
       <c r="B4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" spans="1:14">
       <c r="B5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="B6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="B7" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="B8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="B9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="B10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="B11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -71605,94 +71610,94 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
     </row>
     <row r="2" ht="28" spans="1:4">
       <c r="A2" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D2" s="4"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>292</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>291</v>
       </c>
       <c r="D5" s="4"/>
     </row>
     <row r="6" ht="42" spans="1:4">
       <c r="A6" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="7" ht="42" spans="1:4">
       <c r="A7" s="5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D7" s="4"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="5" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D8" s="4"/>
     </row>
     <row r="9" ht="42" spans="1:4">
       <c r="A9" s="6"/>
       <c r="B9" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" ht="140" spans="1:4">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="7"/>
       <c r="B11" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -71700,7 +71705,7 @@
     <row r="12" spans="1:4">
       <c r="A12" s="7"/>
       <c r="B12" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>

</xml_diff>